<commit_message>
R2 update: Ethan/Carson (7-1) and Wojcio/R.Bass (4-4 draw)
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9336,7 +9336,9 @@
       <c r="D3" s="158" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="205" t="n"/>
+      <c r="E3" s="205" t="n">
+        <v>4</v>
+      </c>
       <c r="F3" s="205" t="n"/>
       <c r="G3" s="205" t="n"/>
       <c r="H3" s="205" t="n"/>
@@ -9345,15 +9347,15 @@
       <c r="K3" s="205" t="n"/>
       <c r="L3" s="160" t="n"/>
       <c r="M3" s="207" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N3" s="205" t="inlineStr">
         <is>
-          <t>0-1-0</t>
+          <t>0-1-1</t>
         </is>
       </c>
       <c r="O3" s="216" t="n">
-        <v>43</v>
+        <v>41.5</v>
       </c>
       <c r="Q3" s="217" t="inlineStr">
         <is>
@@ -9373,7 +9375,9 @@
       <c r="D4" s="162" t="n">
         <v>43</v>
       </c>
-      <c r="E4" s="163" t="n"/>
+      <c r="E4" s="163" t="n">
+        <v>40</v>
+      </c>
       <c r="F4" s="163" t="n"/>
       <c r="G4" s="163" t="n"/>
       <c r="H4" s="163" t="n"/>
@@ -9416,7 +9420,9 @@
       <c r="D5" s="165" t="n">
         <v>6</v>
       </c>
-      <c r="E5" s="166" t="n"/>
+      <c r="E5" s="166" t="n">
+        <v>7</v>
+      </c>
       <c r="F5" s="166" t="n"/>
       <c r="G5" s="166" t="n"/>
       <c r="H5" s="166" t="n"/>
@@ -9425,15 +9431,15 @@
       <c r="K5" s="166" t="n"/>
       <c r="L5" s="167" t="n"/>
       <c r="M5" s="211" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="N5" s="203" t="inlineStr">
         <is>
-          <t>1-0-0</t>
+          <t>2-0-0</t>
         </is>
       </c>
       <c r="O5" s="197" t="n">
-        <v>39</v>
+        <v>37.5</v>
       </c>
       <c r="Q5" s="33" t="n">
         <v>1</v>
@@ -9451,7 +9457,9 @@
       <c r="D6" s="169" t="n">
         <v>39</v>
       </c>
-      <c r="E6" s="170" t="n"/>
+      <c r="E6" s="170" t="n">
+        <v>36</v>
+      </c>
       <c r="F6" s="170" t="n"/>
       <c r="G6" s="170" t="n"/>
       <c r="H6" s="170" t="n"/>
@@ -9484,7 +9492,9 @@
       <c r="D7" s="158" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="205" t="n"/>
+      <c r="E7" s="205" t="n">
+        <v>4</v>
+      </c>
       <c r="F7" s="205" t="n"/>
       <c r="G7" s="205" t="n"/>
       <c r="H7" s="205" t="n"/>
@@ -9493,15 +9503,15 @@
       <c r="K7" s="205" t="n"/>
       <c r="L7" s="160" t="n"/>
       <c r="M7" s="207" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N7" s="205" t="inlineStr">
         <is>
-          <t>0-1-0</t>
+          <t>0-1-1</t>
         </is>
       </c>
       <c r="O7" s="216" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Q7" s="33" t="n">
         <v>3</v>
@@ -9519,7 +9529,9 @@
       <c r="D8" s="162" t="n">
         <v>43</v>
       </c>
-      <c r="E8" s="163" t="n"/>
+      <c r="E8" s="163" t="n">
+        <v>39</v>
+      </c>
       <c r="F8" s="163" t="n"/>
       <c r="G8" s="163" t="n"/>
       <c r="H8" s="163" t="n"/>
@@ -9552,7 +9564,9 @@
       <c r="D9" s="165" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="166" t="n"/>
+      <c r="E9" s="166" t="n">
+        <v>1</v>
+      </c>
       <c r="F9" s="166" t="n"/>
       <c r="G9" s="166" t="n"/>
       <c r="H9" s="166" t="n"/>
@@ -9561,15 +9575,15 @@
       <c r="K9" s="166" t="n"/>
       <c r="L9" s="167" t="n"/>
       <c r="M9" s="211" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N9" s="203" t="inlineStr">
         <is>
-          <t>1-0-0</t>
+          <t>1-1-0</t>
         </is>
       </c>
       <c r="O9" s="197" t="n">
-        <v>38</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="10" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -9582,7 +9596,9 @@
       <c r="D10" s="169" t="n">
         <v>38</v>
       </c>
-      <c r="E10" s="170" t="n"/>
+      <c r="E10" s="170" t="n">
+        <v>47</v>
+      </c>
       <c r="F10" s="170" t="n"/>
       <c r="G10" s="170" t="n"/>
       <c r="H10" s="170" t="n"/>

</xml_diff>

<commit_message>
Process R2 scores: 3 of 7 matches recorded
- Ethan High 7 pts def. Carson Bass 1 pt (NET 36 vs 47)
- Brian Wojcio 4 pts drew Rob Bass 4 pts (NET 40 vs 39)
- Charlotte Hayes 8 pts def. Kaylan Adams 0 pts (NET 42 vs 51)

Standings leaders: Charlotte Hayes 14 pts (2-0-0), Ethan High 13 pts (2-0-0).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9974,7 +9974,9 @@
       <c r="D21" s="165" t="n">
         <v>6</v>
       </c>
-      <c r="E21" s="166" t="n"/>
+      <c r="E21" s="166" t="n">
+        <v>8</v>
+      </c>
       <c r="F21" s="166" t="n"/>
       <c r="G21" s="166" t="n"/>
       <c r="H21" s="166" t="n"/>
@@ -9983,15 +9985,15 @@
       <c r="K21" s="166" t="n"/>
       <c r="L21" s="167" t="n"/>
       <c r="M21" s="211" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="N21" s="203" t="inlineStr">
         <is>
-          <t>1-0-0</t>
+          <t>2-0-0</t>
         </is>
       </c>
       <c r="O21" s="197" t="n">
-        <v>35</v>
+        <v>38.5</v>
       </c>
       <c r="Q21" s="154" t="inlineStr">
         <is>
@@ -10010,7 +10012,9 @@
       <c r="D22" s="169" t="n">
         <v>35</v>
       </c>
-      <c r="E22" s="170" t="n"/>
+      <c r="E22" s="170" t="n">
+        <v>42</v>
+      </c>
       <c r="F22" s="170" t="n"/>
       <c r="G22" s="170" t="n"/>
       <c r="H22" s="170" t="n"/>
@@ -10142,7 +10146,9 @@
       <c r="D27" s="158" t="n">
         <v>4</v>
       </c>
-      <c r="E27" s="205" t="n"/>
+      <c r="E27" s="205" t="n">
+        <v>0</v>
+      </c>
       <c r="F27" s="205" t="n"/>
       <c r="G27" s="205" t="n"/>
       <c r="H27" s="205" t="n"/>
@@ -10155,11 +10161,11 @@
       </c>
       <c r="N27" s="205" t="inlineStr">
         <is>
-          <t>0-0-1</t>
+          <t>0-1-1</t>
         </is>
       </c>
       <c r="O27" s="216" t="n">
-        <v>54</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="28" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -10172,7 +10178,9 @@
       <c r="D28" s="162" t="n">
         <v>54</v>
       </c>
-      <c r="E28" s="163" t="n"/>
+      <c r="E28" s="163" t="n">
+        <v>51</v>
+      </c>
       <c r="F28" s="163" t="n"/>
       <c r="G28" s="163" t="n"/>
       <c r="H28" s="163" t="n"/>

</xml_diff>

<commit_message>
Process R2 scores: 5 of 7 matches recorded
New matches this update:
- Curtis Lynn def. Bruce Atkins 6-2
- David Maddox def. Megan Serian 8-0

Previously recorded R2:
- Ethan High def. Carson Bass 7-1
- Brian Wojcio drew Rob Bass 4-4
- Charlotte Hayes def. Kaylan Adams 8-0

Charlotte Hayes leads at 14 pts; Curtis Lynn and Ethan High
tie at 13 (Curtis gets #2 seed on name tiebreak — identical 2-0-0
and 37.5 avg NET).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9710,7 +9710,9 @@
       <c r="D13" s="165" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="166" t="n"/>
+      <c r="E13" s="166" t="n">
+        <v>2</v>
+      </c>
       <c r="F13" s="166" t="n"/>
       <c r="G13" s="166" t="n"/>
       <c r="H13" s="166" t="n"/>
@@ -9719,15 +9721,15 @@
       <c r="K13" s="166" t="n"/>
       <c r="L13" s="167" t="n"/>
       <c r="M13" s="211" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N13" s="203" t="inlineStr">
         <is>
-          <t>1-0-0</t>
+          <t>1-1-0</t>
         </is>
       </c>
       <c r="O13" s="197" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="R13" s="39" t="inlineStr">
         <is>
@@ -9750,7 +9752,9 @@
       <c r="D14" s="169" t="n">
         <v>33</v>
       </c>
-      <c r="E14" s="170" t="n"/>
+      <c r="E14" s="170" t="n">
+        <v>39</v>
+      </c>
       <c r="F14" s="170" t="n"/>
       <c r="G14" s="170" t="n"/>
       <c r="H14" s="170" t="n"/>
@@ -9836,7 +9840,9 @@
       <c r="D17" s="165" t="n">
         <v>7</v>
       </c>
-      <c r="E17" s="166" t="n"/>
+      <c r="E17" s="166" t="n">
+        <v>6</v>
+      </c>
       <c r="F17" s="166" t="n"/>
       <c r="G17" s="166" t="n"/>
       <c r="H17" s="166" t="n"/>
@@ -9845,15 +9851,15 @@
       <c r="K17" s="166" t="n"/>
       <c r="L17" s="167" t="n"/>
       <c r="M17" s="211" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="N17" s="203" t="inlineStr">
         <is>
-          <t>1-0-0</t>
+          <t>2-0-0</t>
         </is>
       </c>
       <c r="O17" s="197" t="n">
-        <v>37</v>
+        <v>37.5</v>
       </c>
       <c r="Q17" s="212" t="inlineStr">
         <is>
@@ -9871,7 +9877,9 @@
       <c r="D18" s="169" t="n">
         <v>37</v>
       </c>
-      <c r="E18" s="170" t="n"/>
+      <c r="E18" s="170" t="n">
+        <v>38</v>
+      </c>
       <c r="F18" s="170" t="n"/>
       <c r="G18" s="170" t="n"/>
       <c r="H18" s="170" t="n"/>
@@ -10040,7 +10048,9 @@
         </is>
       </c>
       <c r="D23" s="158" t="n"/>
-      <c r="E23" s="205" t="n"/>
+      <c r="E23" s="205" t="n">
+        <v>8</v>
+      </c>
       <c r="F23" s="205" t="n"/>
       <c r="G23" s="205" t="n"/>
       <c r="H23" s="205" t="n"/>
@@ -10048,9 +10058,17 @@
       <c r="J23" s="205" t="n"/>
       <c r="K23" s="205" t="n"/>
       <c r="L23" s="160" t="n"/>
-      <c r="M23" s="207" t="n"/>
-      <c r="N23" s="205" t="n"/>
-      <c r="O23" s="216" t="n"/>
+      <c r="M23" s="207" t="n">
+        <v>8</v>
+      </c>
+      <c r="N23" s="205" t="inlineStr">
+        <is>
+          <t>1-0-0</t>
+        </is>
+      </c>
+      <c r="O23" s="216" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="24" ht="13.5" customHeight="1" s="181" thickBot="1">
       <c r="B24" s="200" t="n"/>
@@ -10060,7 +10078,9 @@
         </is>
       </c>
       <c r="D24" s="162" t="n"/>
-      <c r="E24" s="163" t="n"/>
+      <c r="E24" s="163" t="n">
+        <v>43</v>
+      </c>
       <c r="F24" s="163" t="n"/>
       <c r="G24" s="163" t="n"/>
       <c r="H24" s="163" t="n"/>
@@ -10208,7 +10228,9 @@
       <c r="D29" s="165" t="n">
         <v>7</v>
       </c>
-      <c r="E29" s="166" t="n"/>
+      <c r="E29" s="166" t="n">
+        <v>0</v>
+      </c>
       <c r="F29" s="166" t="n"/>
       <c r="G29" s="166" t="n"/>
       <c r="H29" s="166" t="n"/>
@@ -10221,11 +10243,11 @@
       </c>
       <c r="N29" s="203" t="inlineStr">
         <is>
-          <t>1-0-0</t>
+          <t>1-1-0</t>
         </is>
       </c>
       <c r="O29" s="197" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -10238,7 +10260,9 @@
       <c r="D30" s="169" t="n">
         <v>50</v>
       </c>
-      <c r="E30" s="170" t="n"/>
+      <c r="E30" s="170" t="n">
+        <v>52</v>
+      </c>
       <c r="F30" s="170" t="n"/>
       <c r="G30" s="170" t="n"/>
       <c r="H30" s="170" t="n"/>

</xml_diff>

<commit_message>
Process R2 scores: 6 of 7 matches recorded
New R2 match:
- Ben Linck (8) def. Jerome Martin (0) at Skybrook — NET 36 vs 54

Still outstanding: Michael McHugh vs Alex Palmer.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9913,7 +9913,9 @@
       <c r="D19" s="158" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="205" t="n"/>
+      <c r="E19" s="205" t="n">
+        <v>8</v>
+      </c>
       <c r="F19" s="205" t="n"/>
       <c r="G19" s="205" t="n"/>
       <c r="H19" s="205" t="n"/>
@@ -9922,15 +9924,15 @@
       <c r="K19" s="205" t="n"/>
       <c r="L19" s="160" t="n"/>
       <c r="M19" s="207" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="N19" s="205" t="inlineStr">
         <is>
-          <t>0-1-0</t>
+          <t>1-1-0</t>
         </is>
       </c>
       <c r="O19" s="216" t="n">
-        <v>39</v>
+        <v>37.5</v>
       </c>
       <c r="Q19" s="154" t="inlineStr">
         <is>
@@ -9948,7 +9950,9 @@
       <c r="D20" s="162" t="n">
         <v>39</v>
       </c>
-      <c r="E20" s="163" t="n"/>
+      <c r="E20" s="163" t="n">
+        <v>36</v>
+      </c>
       <c r="F20" s="163" t="n"/>
       <c r="G20" s="163" t="n"/>
       <c r="H20" s="163" t="n"/>
@@ -10108,7 +10112,9 @@
       <c r="D25" s="165" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="166" t="n"/>
+      <c r="E25" s="166" t="n">
+        <v>0</v>
+      </c>
       <c r="F25" s="166" t="n"/>
       <c r="G25" s="166" t="n"/>
       <c r="H25" s="166" t="n"/>
@@ -10121,7 +10127,7 @@
       </c>
       <c r="N25" s="203" t="inlineStr">
         <is>
-          <t>0-0-1</t>
+          <t>0-1-1</t>
         </is>
       </c>
       <c r="O25" s="197" t="n">
@@ -10138,7 +10144,9 @@
       <c r="D26" s="169" t="n">
         <v>54</v>
       </c>
-      <c r="E26" s="170" t="n"/>
+      <c r="E26" s="170" t="n">
+        <v>54</v>
+      </c>
       <c r="F26" s="170" t="n"/>
       <c r="G26" s="170" t="n"/>
       <c r="H26" s="170" t="n"/>

</xml_diff>

<commit_message>
Complete R2: all 7 matches recorded
Final R2 match:
- Michael McHugh (6) def. Alex Palmer (2) at Skybrook — NET 43 vs 49

Round 2 is now complete.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9632,7 +9632,9 @@
       <c r="D11" s="158" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="205" t="n"/>
+      <c r="E11" s="205" t="n">
+        <v>6</v>
+      </c>
       <c r="F11" s="205" t="n"/>
       <c r="G11" s="205" t="n"/>
       <c r="H11" s="205" t="n"/>
@@ -9641,15 +9643,15 @@
       <c r="K11" s="205" t="n"/>
       <c r="L11" s="160" t="n"/>
       <c r="M11" s="207" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N11" s="205" t="inlineStr">
         <is>
-          <t>0-1-0</t>
+          <t>1-1-0</t>
         </is>
       </c>
       <c r="O11" s="216" t="n">
-        <v>46</v>
+        <v>44.5</v>
       </c>
       <c r="R11" s="36" t="inlineStr">
         <is>
@@ -9672,7 +9674,9 @@
       <c r="D12" s="162" t="n">
         <v>46</v>
       </c>
-      <c r="E12" s="163" t="n"/>
+      <c r="E12" s="163" t="n">
+        <v>43</v>
+      </c>
       <c r="F12" s="163" t="n"/>
       <c r="G12" s="163" t="n"/>
       <c r="H12" s="163" t="n"/>
@@ -9782,7 +9786,9 @@
       <c r="D15" s="158" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="205" t="n"/>
+      <c r="E15" s="205" t="n">
+        <v>2</v>
+      </c>
       <c r="F15" s="205" t="n"/>
       <c r="G15" s="205" t="n"/>
       <c r="H15" s="205" t="n"/>
@@ -9791,15 +9797,15 @@
       <c r="K15" s="205" t="n"/>
       <c r="L15" s="160" t="n"/>
       <c r="M15" s="207" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" s="205" t="inlineStr">
         <is>
-          <t>0-1-0</t>
+          <t>0-2-0</t>
         </is>
       </c>
       <c r="O15" s="216" t="n">
-        <v>48</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="16" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -9812,7 +9818,9 @@
       <c r="D16" s="162" t="n">
         <v>48</v>
       </c>
-      <c r="E16" s="163" t="n"/>
+      <c r="E16" s="163" t="n">
+        <v>49</v>
+      </c>
       <c r="F16" s="163" t="n"/>
       <c r="G16" s="163" t="n"/>
       <c r="H16" s="163" t="n"/>

</xml_diff>

<commit_message>
Process R3 scores: 2 of 7 matches recorded
Matches:
- Curtis Lynn def. Nick Coglianese, 8-0 (NET 37 vs 54)
- Alex Palmer def. Kaylan Adams, 7-1 (NET 39 vs 54)

Curtis Lynn moves to 3-0-0 and takes the top seed at 21 pts.
Alex Palmer earns his first win of the season.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9789,7 +9789,9 @@
       <c r="E15" s="205" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="205" t="n"/>
+      <c r="F15" s="205" t="n">
+        <v>7</v>
+      </c>
       <c r="G15" s="205" t="n"/>
       <c r="H15" s="205" t="n"/>
       <c r="I15" s="205" t="n"/>
@@ -9797,15 +9799,15 @@
       <c r="K15" s="205" t="n"/>
       <c r="L15" s="160" t="n"/>
       <c r="M15" s="207" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="N15" s="205" t="inlineStr">
         <is>
-          <t>0-2-0</t>
+          <t>1-2-0</t>
         </is>
       </c>
       <c r="O15" s="216" t="n">
-        <v>48.5</v>
+        <v>45.3</v>
       </c>
     </row>
     <row r="16" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -9821,7 +9823,9 @@
       <c r="E16" s="163" t="n">
         <v>49</v>
       </c>
-      <c r="F16" s="163" t="n"/>
+      <c r="F16" s="163" t="n">
+        <v>39</v>
+      </c>
       <c r="G16" s="163" t="n"/>
       <c r="H16" s="163" t="n"/>
       <c r="I16" s="163" t="n"/>
@@ -9851,7 +9855,9 @@
       <c r="E17" s="166" t="n">
         <v>6</v>
       </c>
-      <c r="F17" s="166" t="n"/>
+      <c r="F17" s="166" t="n">
+        <v>8</v>
+      </c>
       <c r="G17" s="166" t="n"/>
       <c r="H17" s="166" t="n"/>
       <c r="I17" s="166" t="n"/>
@@ -9859,15 +9865,15 @@
       <c r="K17" s="166" t="n"/>
       <c r="L17" s="167" t="n"/>
       <c r="M17" s="211" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="N17" s="203" t="inlineStr">
         <is>
-          <t>2-0-0</t>
+          <t>3-0-0</t>
         </is>
       </c>
       <c r="O17" s="197" t="n">
-        <v>37.5</v>
+        <v>37.3</v>
       </c>
       <c r="Q17" s="212" t="inlineStr">
         <is>
@@ -9888,7 +9894,9 @@
       <c r="E18" s="170" t="n">
         <v>38</v>
       </c>
-      <c r="F18" s="170" t="n"/>
+      <c r="F18" s="170" t="n">
+        <v>37</v>
+      </c>
       <c r="G18" s="170" t="n"/>
       <c r="H18" s="170" t="n"/>
       <c r="I18" s="170" t="n"/>
@@ -10185,7 +10193,9 @@
       <c r="E27" s="205" t="n">
         <v>0</v>
       </c>
-      <c r="F27" s="205" t="n"/>
+      <c r="F27" s="205" t="n">
+        <v>1</v>
+      </c>
       <c r="G27" s="205" t="n"/>
       <c r="H27" s="205" t="n"/>
       <c r="I27" s="205" t="n"/>
@@ -10193,15 +10203,15 @@
       <c r="K27" s="205" t="n"/>
       <c r="L27" s="160" t="n"/>
       <c r="M27" s="207" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N27" s="205" t="inlineStr">
         <is>
-          <t>0-1-1</t>
+          <t>0-2-1</t>
         </is>
       </c>
       <c r="O27" s="216" t="n">
-        <v>52.5</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -10217,7 +10227,9 @@
       <c r="E28" s="163" t="n">
         <v>51</v>
       </c>
-      <c r="F28" s="163" t="n"/>
+      <c r="F28" s="163" t="n">
+        <v>54</v>
+      </c>
       <c r="G28" s="163" t="n"/>
       <c r="H28" s="163" t="n"/>
       <c r="I28" s="163" t="n"/>
@@ -10307,7 +10319,9 @@
         <v>1</v>
       </c>
       <c r="E31" s="205" t="n"/>
-      <c r="F31" s="205" t="n"/>
+      <c r="F31" s="205" t="n">
+        <v>0</v>
+      </c>
       <c r="G31" s="205" t="n"/>
       <c r="H31" s="205" t="n"/>
       <c r="I31" s="205" t="n"/>
@@ -10319,11 +10333,11 @@
       </c>
       <c r="N31" s="205" t="inlineStr">
         <is>
-          <t>0-1-0</t>
+          <t>0-2-0</t>
         </is>
       </c>
       <c r="O31" s="216" t="n">
-        <v>53</v>
+        <v>53.5</v>
       </c>
     </row>
     <row r="32" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -10337,7 +10351,9 @@
         <v>53</v>
       </c>
       <c r="E32" s="163" t="n"/>
-      <c r="F32" s="163" t="n"/>
+      <c r="F32" s="163" t="n">
+        <v>54</v>
+      </c>
       <c r="G32" s="163" t="n"/>
       <c r="H32" s="163" t="n"/>
       <c r="I32" s="163" t="n"/>

</xml_diff>

<commit_message>
R3: Ben Linck d. Megan Serian 4.5-3.5 at Highland Creek
R3 matches recorded (3 of 7):
- Curtis Lynn d. Nick Coglianese 8-0
- Alex Palmer d. Kaylan Adams 7-1
- Ben Linck d. Megan Serian 4.5-3.5 (new)

Curtis Lynn holds top seed at 21 pts (3-0-0). Ben Linck climbs to #2
at 14.5 pts after his R3 win over Megan.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9932,7 +9932,9 @@
       <c r="E19" s="205" t="n">
         <v>8</v>
       </c>
-      <c r="F19" s="205" t="n"/>
+      <c r="F19" s="205" t="n">
+        <v>4.5</v>
+      </c>
       <c r="G19" s="205" t="n"/>
       <c r="H19" s="205" t="n"/>
       <c r="I19" s="205" t="n"/>
@@ -9940,15 +9942,15 @@
       <c r="K19" s="205" t="n"/>
       <c r="L19" s="160" t="n"/>
       <c r="M19" s="207" t="n">
-        <v>10</v>
+        <v>14.5</v>
       </c>
       <c r="N19" s="205" t="inlineStr">
         <is>
-          <t>1-1-0</t>
+          <t>2-1-0</t>
         </is>
       </c>
       <c r="O19" s="216" t="n">
-        <v>37.5</v>
+        <v>39</v>
       </c>
       <c r="Q19" s="154" t="inlineStr">
         <is>
@@ -9969,7 +9971,9 @@
       <c r="E20" s="163" t="n">
         <v>36</v>
       </c>
-      <c r="F20" s="163" t="n"/>
+      <c r="F20" s="163" t="n">
+        <v>42</v>
+      </c>
       <c r="G20" s="163" t="n"/>
       <c r="H20" s="163" t="n"/>
       <c r="I20" s="163" t="n"/>
@@ -10259,7 +10263,9 @@
       <c r="E29" s="166" t="n">
         <v>0</v>
       </c>
-      <c r="F29" s="166" t="n"/>
+      <c r="F29" s="166" t="n">
+        <v>3.5</v>
+      </c>
       <c r="G29" s="166" t="n"/>
       <c r="H29" s="166" t="n"/>
       <c r="I29" s="166" t="n"/>
@@ -10267,15 +10273,15 @@
       <c r="K29" s="166" t="n"/>
       <c r="L29" s="167" t="n"/>
       <c r="M29" s="211" t="n">
-        <v>7</v>
+        <v>10.5</v>
       </c>
       <c r="N29" s="203" t="inlineStr">
         <is>
-          <t>1-1-0</t>
+          <t>1-2-0</t>
         </is>
       </c>
       <c r="O29" s="197" t="n">
-        <v>51</v>
+        <v>48.3</v>
       </c>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -10291,7 +10297,9 @@
       <c r="E30" s="170" t="n">
         <v>52</v>
       </c>
-      <c r="F30" s="170" t="n"/>
+      <c r="F30" s="170" t="n">
+        <v>43</v>
+      </c>
       <c r="G30" s="170" t="n"/>
       <c r="H30" s="170" t="n"/>
       <c r="I30" s="170" t="n"/>

</xml_diff>

<commit_message>
R3: David Maddox d. Jerome Martin 7-1 at Skybrook
R3 now 4 of 7 matches recorded. David Maddox up to 15 pts (2-0-0), moves to seed 2. Standings re-sorted.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -10075,7 +10075,9 @@
       <c r="E23" s="205" t="n">
         <v>8</v>
       </c>
-      <c r="F23" s="205" t="n"/>
+      <c r="F23" s="205" t="n">
+        <v>7</v>
+      </c>
       <c r="G23" s="205" t="n"/>
       <c r="H23" s="205" t="n"/>
       <c r="I23" s="205" t="n"/>
@@ -10083,15 +10085,15 @@
       <c r="K23" s="205" t="n"/>
       <c r="L23" s="160" t="n"/>
       <c r="M23" s="207" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="N23" s="205" t="inlineStr">
         <is>
-          <t>1-0-0</t>
+          <t>2-0-0</t>
         </is>
       </c>
       <c r="O23" s="216" t="n">
-        <v>43</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="24" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -10105,7 +10107,9 @@
       <c r="E24" s="163" t="n">
         <v>43</v>
       </c>
-      <c r="F24" s="163" t="n"/>
+      <c r="F24" s="163" t="n">
+        <v>52</v>
+      </c>
       <c r="G24" s="163" t="n"/>
       <c r="H24" s="163" t="n"/>
       <c r="I24" s="163" t="n"/>
@@ -10135,7 +10139,9 @@
       <c r="E25" s="166" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="166" t="n"/>
+      <c r="F25" s="166" t="n">
+        <v>1</v>
+      </c>
       <c r="G25" s="166" t="n"/>
       <c r="H25" s="166" t="n"/>
       <c r="I25" s="166" t="n"/>
@@ -10143,11 +10149,11 @@
       <c r="K25" s="166" t="n"/>
       <c r="L25" s="167" t="n"/>
       <c r="M25" s="211" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N25" s="203" t="inlineStr">
         <is>
-          <t>0-1-1</t>
+          <t>0-2-1</t>
         </is>
       </c>
       <c r="O25" s="197" t="n">
@@ -10167,7 +10173,9 @@
       <c r="E26" s="170" t="n">
         <v>54</v>
       </c>
-      <c r="F26" s="170" t="n"/>
+      <c r="F26" s="170" t="n">
+        <v>54</v>
+      </c>
       <c r="G26" s="170" t="n"/>
       <c r="H26" s="170" t="n"/>
       <c r="I26" s="170" t="n"/>

</xml_diff>

<commit_message>
R4 update: Maddox–Coglianese draw recorded
Round 4 opener (1 of 7 matches in):
- David Maddox vs Nick Coglianese: 4-4 draw, both NET 43

Standings: Maddox up to 19 pts (2-0-1), holds seed #2; Nick to 5 pts
(0-2-1), seed #12. Curtis Lynn still leads at 21 pts.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -10078,22 +10078,24 @@
       <c r="F23" s="205" t="n">
         <v>7</v>
       </c>
-      <c r="G23" s="205" t="n"/>
+      <c r="G23" s="205" t="n">
+        <v>4</v>
+      </c>
       <c r="H23" s="205" t="n"/>
       <c r="I23" s="205" t="n"/>
       <c r="J23" s="205" t="n"/>
       <c r="K23" s="205" t="n"/>
       <c r="L23" s="160" t="n"/>
       <c r="M23" s="207" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="N23" s="205" t="inlineStr">
         <is>
-          <t>2-0-0</t>
+          <t>2-0-1</t>
         </is>
       </c>
       <c r="O23" s="216" t="n">
-        <v>47.5</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -10110,7 +10112,9 @@
       <c r="F24" s="163" t="n">
         <v>52</v>
       </c>
-      <c r="G24" s="163" t="n"/>
+      <c r="G24" s="163" t="n">
+        <v>43</v>
+      </c>
       <c r="H24" s="163" t="n"/>
       <c r="I24" s="163" t="n"/>
       <c r="J24" s="163" t="n"/>
@@ -10338,22 +10342,24 @@
       <c r="F31" s="205" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="205" t="n"/>
+      <c r="G31" s="205" t="n">
+        <v>4</v>
+      </c>
       <c r="H31" s="205" t="n"/>
       <c r="I31" s="205" t="n"/>
       <c r="J31" s="205" t="n"/>
       <c r="K31" s="205" t="n"/>
       <c r="L31" s="160" t="n"/>
       <c r="M31" s="207" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N31" s="205" t="inlineStr">
         <is>
-          <t>0-2-0</t>
+          <t>0-2-1</t>
         </is>
       </c>
       <c r="O31" s="216" t="n">
-        <v>53.5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" ht="13.5" customHeight="1" s="181" thickBot="1">
@@ -10370,7 +10376,9 @@
       <c r="F32" s="163" t="n">
         <v>54</v>
       </c>
-      <c r="G32" s="163" t="n"/>
+      <c r="G32" s="163" t="n">
+        <v>43</v>
+      </c>
       <c r="H32" s="163" t="n"/>
       <c r="I32" s="163" t="n"/>
       <c r="J32" s="163" t="n"/>

</xml_diff>

<commit_message>
R4 makeup: Charlotte Hayes def. Megan Serian 8-0
R4 matches now recorded (3 of 7):
- David Maddox 4-4 Nick Coglianese (draw)
- Ethan High def. Alex Palmer 7-1
- Charlotte Hayes def. Megan Serian 8-0 (NET 41 vs 54) at Highland Creek

Standings: Charlotte takes over #1 at 22 pts (3-0-0), ahead of Curtis Lynn
(21) and Ethan High (20). Megan falls to 10.5 pts (1-3-0). Bruce overrides
re-applied; currentRound restored to 5.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -10018,22 +10018,24 @@
         <v>8</v>
       </c>
       <c r="F21" s="166" t="n"/>
-      <c r="G21" s="166" t="n"/>
+      <c r="G21" s="166" t="n">
+        <v>8</v>
+      </c>
       <c r="H21" s="166" t="n"/>
       <c r="I21" s="166" t="n"/>
       <c r="J21" s="166" t="n"/>
       <c r="K21" s="166" t="n"/>
       <c r="L21" s="167" t="n"/>
       <c r="M21" s="226" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="N21" s="218" t="inlineStr">
         <is>
-          <t>2-0-0</t>
+          <t>3-0-0</t>
         </is>
       </c>
       <c r="O21" s="212" t="n">
-        <v>38.5</v>
+        <v>39.3</v>
       </c>
       <c r="Q21" s="154" t="inlineStr">
         <is>
@@ -10056,7 +10058,9 @@
         <v>42</v>
       </c>
       <c r="F22" s="170" t="n"/>
-      <c r="G22" s="170" t="n"/>
+      <c r="G22" s="170" t="n">
+        <v>41</v>
+      </c>
       <c r="H22" s="170" t="n"/>
       <c r="I22" s="170" t="n"/>
       <c r="J22" s="170" t="n"/>
@@ -10286,7 +10290,9 @@
       <c r="F29" s="166" t="n">
         <v>3.5</v>
       </c>
-      <c r="G29" s="166" t="n"/>
+      <c r="G29" s="166" t="n">
+        <v>0</v>
+      </c>
       <c r="H29" s="166" t="n"/>
       <c r="I29" s="166" t="n"/>
       <c r="J29" s="166" t="n"/>
@@ -10297,11 +10303,11 @@
       </c>
       <c r="N29" s="218" t="inlineStr">
         <is>
-          <t>1-2-0</t>
+          <t>1-3-0</t>
         </is>
       </c>
       <c r="O29" s="212" t="n">
-        <v>48.3</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="197" thickBot="1">
@@ -10320,7 +10326,9 @@
       <c r="F30" s="170" t="n">
         <v>43</v>
       </c>
-      <c r="G30" s="170" t="n"/>
+      <c r="G30" s="170" t="n">
+        <v>54</v>
+      </c>
       <c r="H30" s="170" t="n"/>
       <c r="I30" s="170" t="n"/>
       <c r="J30" s="170" t="n"/>

</xml_diff>

<commit_message>
Scores: R3 Brian Wojcio def. Carson Bass 8-0 (Warrior GC)
- R3 makeup @ Warrior Golf Club: Brian Wojcio 8 pts (NET 34) def. Carson Bass 0 pts (NET 47)
- R3 now 6 of 7 recorded (outstanding: Rob Bass vs Bruce replacement)
- Standings: Brian Wojcio up to #6 (14 pts, 1-1-1); Carson Bass 1-2-0

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9342,7 +9342,9 @@
       <c r="E3" s="200" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="200" t="n"/>
+      <c r="F3" s="200" t="n">
+        <v>8</v>
+      </c>
       <c r="G3" s="200" t="n"/>
       <c r="H3" s="200" t="n"/>
       <c r="I3" s="200" t="n"/>
@@ -9350,15 +9352,15 @@
       <c r="K3" s="200" t="n"/>
       <c r="L3" s="160" t="n"/>
       <c r="M3" s="202" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="N3" s="200" t="inlineStr">
         <is>
-          <t>0-1-1</t>
+          <t>1-1-1</t>
         </is>
       </c>
       <c r="O3" s="208" t="n">
-        <v>41.5</v>
+        <v>39</v>
       </c>
       <c r="Q3" s="209" t="inlineStr">
         <is>
@@ -9381,7 +9383,9 @@
       <c r="E4" s="163" t="n">
         <v>40</v>
       </c>
-      <c r="F4" s="163" t="n"/>
+      <c r="F4" s="163" t="n">
+        <v>34</v>
+      </c>
       <c r="G4" s="163" t="n"/>
       <c r="H4" s="163" t="n"/>
       <c r="I4" s="163" t="n"/>
@@ -9578,7 +9582,9 @@
       <c r="E9" s="166" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="166" t="n"/>
+      <c r="F9" s="166" t="n">
+        <v>0</v>
+      </c>
       <c r="G9" s="166" t="n"/>
       <c r="H9" s="166" t="n"/>
       <c r="I9" s="166" t="n"/>
@@ -9590,11 +9596,11 @@
       </c>
       <c r="N9" s="199" t="inlineStr">
         <is>
-          <t>1-1-0</t>
+          <t>1-2-0</t>
         </is>
       </c>
       <c r="O9" s="196" t="n">
-        <v>42.5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" ht="13.5" customHeight="1" s="219" thickBot="1">
@@ -9610,7 +9616,9 @@
       <c r="E10" s="170" t="n">
         <v>47</v>
       </c>
-      <c r="F10" s="170" t="n"/>
+      <c r="F10" s="170" t="n">
+        <v>47</v>
+      </c>
       <c r="G10" s="170" t="n"/>
       <c r="H10" s="170" t="n"/>
       <c r="I10" s="170" t="n"/>

</xml_diff>

<commit_message>
R5: Curtis Lynn def. Preston Stoner 8-0 (Skybrook) — Curtis takes #1 seed
New R5 makeup match recorded (Skybrook, NET 35 vs 44):
- Curtis Lynn def. Preston Stoner 8-0

Curtis Lynn: 21 -> 29 pts, 4-0-0, avg NET 36.8 — now the top seed
over Ethan High (27, 4-0-0). Preston takes his first loss (3-2-0),
points unchanged at 22.5. R5 now 3 of 6 recorded.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9898,21 +9898,23 @@
         <v>8</v>
       </c>
       <c r="G17" s="166" t="n"/>
-      <c r="H17" s="166" t="n"/>
+      <c r="H17" s="166" t="n">
+        <v>8</v>
+      </c>
       <c r="I17" s="166" t="n"/>
       <c r="J17" s="166" t="n"/>
       <c r="K17" s="166" t="n"/>
       <c r="L17" s="167" t="n"/>
       <c r="M17" s="226" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="N17" s="218" t="inlineStr">
         <is>
-          <t>3-0-0</t>
+          <t>4-0-0</t>
         </is>
       </c>
       <c r="O17" s="212" t="n">
-        <v>37.3</v>
+        <v>36.8</v>
       </c>
       <c r="Q17" s="227" t="inlineStr">
         <is>
@@ -9937,7 +9939,9 @@
         <v>37</v>
       </c>
       <c r="G18" s="170" t="n"/>
-      <c r="H18" s="170" t="n"/>
+      <c r="H18" s="170" t="n">
+        <v>35</v>
+      </c>
       <c r="I18" s="170" t="n"/>
       <c r="J18" s="170" t="n"/>
       <c r="K18" s="170" t="n"/>
@@ -9977,7 +9981,9 @@
       <c r="G19" s="220" t="n">
         <v>8</v>
       </c>
-      <c r="H19" s="220" t="n"/>
+      <c r="H19" s="220" t="n">
+        <v>0</v>
+      </c>
       <c r="I19" s="220" t="n"/>
       <c r="J19" s="220" t="n"/>
       <c r="K19" s="220" t="n"/>
@@ -9987,11 +9993,11 @@
       </c>
       <c r="N19" s="220" t="inlineStr">
         <is>
-          <t>3-1-0</t>
+          <t>3-2-0</t>
         </is>
       </c>
       <c r="O19" s="230" t="n">
-        <v>38.8</v>
+        <v>39.8</v>
       </c>
       <c r="Q19" s="154" t="inlineStr">
         <is>
@@ -10018,7 +10024,9 @@
       <c r="G20" s="163" t="n">
         <v>38</v>
       </c>
-      <c r="H20" s="163" t="n"/>
+      <c r="H20" s="163" t="n">
+        <v>44</v>
+      </c>
       <c r="I20" s="163" t="n"/>
       <c r="J20" s="163" t="n"/>
       <c r="K20" s="163" t="n"/>

</xml_diff>

<commit_message>
R6: Nick Coglianese def. Kaylan Adams 6-2 (Highland Creek)
New R6 match recorded (Highland Creek, NET 45 vs 50):
- Nick Coglianese def. Kaylan Adams 6-2

Nick: 7 -> 13 pts, first win of the season (0-3-1 -> 1-3-1), avg NET
51.0 -> 49.8. Kaylan: 12 -> 14 pts, takes the loss (1-3-1 -> 1-4-1).
Seeds reshuffle: Kaylan 7, Carson 8, Nick 9 (Carson over Nick on wins).
R6 now 1 of 6; R3-R5 makeups still open.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -10277,20 +10277,22 @@
       <c r="H27" s="220" t="n">
         <v>7</v>
       </c>
-      <c r="I27" s="220" t="n"/>
+      <c r="I27" s="220" t="n">
+        <v>2</v>
+      </c>
       <c r="J27" s="220" t="n"/>
       <c r="K27" s="220" t="n"/>
       <c r="L27" s="160" t="n"/>
       <c r="M27" s="222" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N27" s="220" t="inlineStr">
         <is>
-          <t>1-3-1</t>
+          <t>1-4-1</t>
         </is>
       </c>
       <c r="O27" s="230" t="n">
-        <v>51.4</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="28" ht="13.5" customHeight="1" s="197" thickBot="1">
@@ -10315,7 +10317,9 @@
       <c r="H28" s="163" t="n">
         <v>48</v>
       </c>
-      <c r="I28" s="163" t="n"/>
+      <c r="I28" s="163" t="n">
+        <v>50</v>
+      </c>
       <c r="J28" s="163" t="n"/>
       <c r="K28" s="163" t="n"/>
       <c r="L28" s="164" t="n"/>
@@ -10423,20 +10427,22 @@
       <c r="H31" s="220" t="n">
         <v>2</v>
       </c>
-      <c r="I31" s="220" t="n"/>
+      <c r="I31" s="220" t="n">
+        <v>6</v>
+      </c>
       <c r="J31" s="220" t="n"/>
       <c r="K31" s="220" t="n"/>
       <c r="L31" s="160" t="n"/>
       <c r="M31" s="222" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="N31" s="220" t="inlineStr">
         <is>
-          <t>0-3-1</t>
+          <t>1-3-1</t>
         </is>
       </c>
       <c r="O31" s="230" t="n">
-        <v>51</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="32" ht="13.5" customHeight="1" s="197" thickBot="1">
@@ -10459,7 +10465,9 @@
       <c r="H32" s="163" t="n">
         <v>54</v>
       </c>
-      <c r="I32" s="163" t="n"/>
+      <c r="I32" s="163" t="n">
+        <v>45</v>
+      </c>
       <c r="J32" s="163" t="n"/>
       <c r="K32" s="163" t="n"/>
       <c r="L32" s="164" t="n"/>

</xml_diff>

<commit_message>
R6: Ethan High def. Rob Bass 5-3 | R8: Ethan High def. Curtis Lynn 7-1
R6 Skybrook  - Ethan High 5, Rob Bass 3      (NET 37 vs 38)
R8 Skybrook  - Ethan High 7, Curtis Lynn 1   (NET 33 vs 40)

Ethan takes the top seed from Curtis Lynn: 39 pts on 6-0-0, avg NET 37.0.
Curtis drops to second at 30 pts and takes his first loss of the season.
Rob Bass falls to 8 pts at 0-2-1.

R6 now 2 of 6 recorded; R8 1 of 7 (played ahead of its Sep 14 window).
R3-R5 makeup matches still outstanding.

Standings verified against the Scores 2026 tab - totals, records, avg NET,
and seed order all reconcile, withdrawn players unseeded.
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -9441,20 +9441,24 @@
         <v>7</v>
       </c>
       <c r="H5" s="166" t="n"/>
-      <c r="I5" s="166" t="n"/>
+      <c r="I5" s="166" t="n">
+        <v>5</v>
+      </c>
       <c r="J5" s="166" t="n"/>
-      <c r="K5" s="166" t="n"/>
+      <c r="K5" s="166" t="n">
+        <v>7</v>
+      </c>
       <c r="L5" s="167" t="n"/>
       <c r="M5" s="226" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="N5" s="218" t="inlineStr">
         <is>
-          <t>4-0-0</t>
+          <t>6-0-0</t>
         </is>
       </c>
       <c r="O5" s="212" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="Q5" s="33" t="n">
         <v>1</v>
@@ -9482,9 +9486,13 @@
         <v>42</v>
       </c>
       <c r="H6" s="170" t="n"/>
-      <c r="I6" s="170" t="n"/>
+      <c r="I6" s="170" t="n">
+        <v>37</v>
+      </c>
       <c r="J6" s="170" t="n"/>
-      <c r="K6" s="170" t="n"/>
+      <c r="K6" s="170" t="n">
+        <v>33</v>
+      </c>
       <c r="L6" s="171" t="n"/>
       <c r="M6" s="223" t="n"/>
       <c r="N6" s="219" t="n"/>
@@ -9517,20 +9525,22 @@
       <c r="F7" s="220" t="n"/>
       <c r="G7" s="220" t="n"/>
       <c r="H7" s="220" t="n"/>
-      <c r="I7" s="220" t="n"/>
+      <c r="I7" s="220" t="n">
+        <v>3</v>
+      </c>
       <c r="J7" s="220" t="n"/>
       <c r="K7" s="220" t="n"/>
       <c r="L7" s="160" t="n"/>
       <c r="M7" s="222" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N7" s="220" t="inlineStr">
         <is>
-          <t>0-1-1</t>
+          <t>0-2-1</t>
         </is>
       </c>
       <c r="O7" s="230" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="Q7" s="33" t="n">
         <v>3</v>
@@ -9554,7 +9564,9 @@
       <c r="F8" s="163" t="n"/>
       <c r="G8" s="163" t="n"/>
       <c r="H8" s="163" t="n"/>
-      <c r="I8" s="163" t="n"/>
+      <c r="I8" s="163" t="n">
+        <v>38</v>
+      </c>
       <c r="J8" s="163" t="n"/>
       <c r="K8" s="163" t="n"/>
       <c r="L8" s="164" t="n"/>
@@ -9903,18 +9915,20 @@
       </c>
       <c r="I17" s="166" t="n"/>
       <c r="J17" s="166" t="n"/>
-      <c r="K17" s="166" t="n"/>
+      <c r="K17" s="166" t="n">
+        <v>1</v>
+      </c>
       <c r="L17" s="167" t="n"/>
       <c r="M17" s="226" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N17" s="218" t="inlineStr">
         <is>
-          <t>4-0-0</t>
+          <t>4-1-0</t>
         </is>
       </c>
       <c r="O17" s="212" t="n">
-        <v>36.8</v>
+        <v>37.4</v>
       </c>
       <c r="Q17" s="227" t="inlineStr">
         <is>
@@ -9944,7 +9958,9 @@
       </c>
       <c r="I18" s="170" t="n"/>
       <c r="J18" s="170" t="n"/>
-      <c r="K18" s="170" t="n"/>
+      <c r="K18" s="170" t="n">
+        <v>40</v>
+      </c>
       <c r="L18" s="171" t="n"/>
       <c r="M18" s="223" t="n"/>
       <c r="N18" s="219" t="n"/>

</xml_diff>

<commit_message>
R8: Charlotte Hayes def. Jerome Martin 6-2 (Highland Creek, NET 39 vs 50)
Charlotte moves to 28 pts / 4-0-0 and takes the #3 seed from Preston Stoner.
Jerome to 13 pts / 1-3-1, seed 10 in a three-way 13-pt tie at 13 pts.
R8 now 2 of 7 recorded (played early).
</commit_message>
<xml_diff>
--- a/2026 IMI Golf League.xlsx
+++ b/2026 IMI Golf League.xlsx
@@ -10083,18 +10083,20 @@
       <c r="H21" s="166" t="n"/>
       <c r="I21" s="166" t="n"/>
       <c r="J21" s="166" t="n"/>
-      <c r="K21" s="166" t="n"/>
+      <c r="K21" s="166" t="n">
+        <v>6</v>
+      </c>
       <c r="L21" s="167" t="n"/>
       <c r="M21" s="226" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="N21" s="218" t="inlineStr">
         <is>
-          <t>3-0-0</t>
+          <t>4-0-0</t>
         </is>
       </c>
       <c r="O21" s="212" t="n">
-        <v>39.3</v>
+        <v>39.2</v>
       </c>
       <c r="Q21" s="154" t="inlineStr">
         <is>
@@ -10123,7 +10125,9 @@
       <c r="H22" s="170" t="n"/>
       <c r="I22" s="170" t="n"/>
       <c r="J22" s="170" t="n"/>
-      <c r="K22" s="170" t="n"/>
+      <c r="K22" s="170" t="n">
+        <v>39</v>
+      </c>
       <c r="L22" s="171" t="n"/>
       <c r="M22" s="223" t="n"/>
       <c r="N22" s="219" t="n"/>
@@ -10223,18 +10227,20 @@
       </c>
       <c r="I25" s="166" t="n"/>
       <c r="J25" s="166" t="n"/>
-      <c r="K25" s="166" t="n"/>
+      <c r="K25" s="166" t="n">
+        <v>2</v>
+      </c>
       <c r="L25" s="167" t="n"/>
       <c r="M25" s="226" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N25" s="218" t="inlineStr">
         <is>
-          <t>1-2-1</t>
+          <t>1-3-1</t>
         </is>
       </c>
       <c r="O25" s="212" t="n">
-        <v>53.5</v>
+        <v>52.8</v>
       </c>
     </row>
     <row r="26" ht="13.5" customHeight="1" s="197" thickBot="1">
@@ -10259,7 +10265,9 @@
       </c>
       <c r="I26" s="170" t="n"/>
       <c r="J26" s="170" t="n"/>
-      <c r="K26" s="170" t="n"/>
+      <c r="K26" s="170" t="n">
+        <v>50</v>
+      </c>
       <c r="L26" s="171" t="n"/>
       <c r="M26" s="223" t="n"/>
       <c r="N26" s="219" t="n"/>

</xml_diff>